<commit_message>
Add contoller, Layout & changes in UI pages
</commit_message>
<xml_diff>
--- a/Week_8/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_8/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="77">
   <si>
     <t>Week_1</t>
   </si>
@@ -237,6 +237,12 @@
   <si>
     <t>Create Contact US Page UI</t>
   </si>
+  <si>
+    <t>Solve Error for find doctor Page + create Doctor Profile pages for 5 Doctors</t>
+  </si>
+  <si>
+    <t>Services Page UI Connect with Services page and department pages (Controller + model)</t>
+  </si>
 </sst>
 </file>
 
@@ -389,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="80">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -609,7 +615,15 @@
     <xf borderId="1" fillId="9" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="9" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="9" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -828,7 +842,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="10.0"/>
-    <col customWidth="1" min="2" max="2" width="62.25"/>
+    <col customWidth="1" min="2" max="2" width="67.5"/>
     <col customWidth="1" min="3" max="3" width="12.25"/>
     <col customWidth="1" min="4" max="4" width="12.13"/>
   </cols>
@@ -4153,9 +4167,15 @@
     </row>
     <row r="99">
       <c r="A99" s="74"/>
-      <c r="B99" s="76"/>
-      <c r="C99" s="71"/>
-      <c r="D99" s="75"/>
+      <c r="B99" s="76" t="s">
+        <v>75</v>
+      </c>
+      <c r="C99" s="73">
+        <v>46089.0</v>
+      </c>
+      <c r="D99" s="75">
+        <v>3.75</v>
+      </c>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
       <c r="G99" s="3"/>
@@ -4181,10 +4201,16 @@
       <c r="AA99" s="3"/>
     </row>
     <row r="100">
-      <c r="A100" s="77"/>
-      <c r="B100" s="77"/>
-      <c r="C100" s="77"/>
-      <c r="D100" s="77"/>
+      <c r="A100" s="74"/>
+      <c r="B100" s="76" t="s">
+        <v>76</v>
+      </c>
+      <c r="C100" s="73">
+        <v>46089.0</v>
+      </c>
+      <c r="D100" s="75">
+        <v>4.15</v>
+      </c>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
       <c r="G100" s="3"/>
@@ -4210,15 +4236,10 @@
       <c r="AA100" s="3"/>
     </row>
     <row r="101">
-      <c r="A101" s="45"/>
-      <c r="B101" s="46" t="s">
-        <v>15</v>
-      </c>
+      <c r="A101" s="77"/>
+      <c r="B101" s="78"/>
       <c r="C101" s="47"/>
-      <c r="D101" s="41">
-        <f>sum(D91:D96)</f>
-        <v>12.9</v>
-      </c>
+      <c r="D101" s="79"/>
       <c r="E101" s="3"/>
       <c r="F101" s="3"/>
       <c r="G101" s="3"/>
@@ -4244,10 +4265,15 @@
       <c r="AA101" s="3"/>
     </row>
     <row r="102">
-      <c r="A102" s="3"/>
-      <c r="B102" s="3"/>
-      <c r="C102" s="3"/>
-      <c r="D102" s="3"/>
+      <c r="A102" s="45"/>
+      <c r="B102" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C102" s="47"/>
+      <c r="D102" s="41">
+        <f>sum(D91:D100)</f>
+        <v>22.7</v>
+      </c>
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
       <c r="G102" s="3"/>
@@ -29096,6 +29122,35 @@
       <c r="Z958" s="3"/>
       <c r="AA958" s="3"/>
     </row>
+    <row r="959">
+      <c r="A959" s="3"/>
+      <c r="B959" s="3"/>
+      <c r="C959" s="3"/>
+      <c r="D959" s="3"/>
+      <c r="E959" s="3"/>
+      <c r="F959" s="3"/>
+      <c r="G959" s="3"/>
+      <c r="H959" s="3"/>
+      <c r="I959" s="3"/>
+      <c r="J959" s="3"/>
+      <c r="K959" s="3"/>
+      <c r="L959" s="3"/>
+      <c r="M959" s="3"/>
+      <c r="N959" s="3"/>
+      <c r="O959" s="3"/>
+      <c r="P959" s="3"/>
+      <c r="Q959" s="3"/>
+      <c r="R959" s="3"/>
+      <c r="S959" s="3"/>
+      <c r="T959" s="3"/>
+      <c r="U959" s="3"/>
+      <c r="V959" s="3"/>
+      <c r="W959" s="3"/>
+      <c r="X959" s="3"/>
+      <c r="Y959" s="3"/>
+      <c r="Z959" s="3"/>
+      <c r="AA959" s="3"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Integrate doctor profile and booking flow & Databse connection + Dynamic Pages
</commit_message>
<xml_diff>
--- a/Week_8/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_8/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="80">
   <si>
     <t>Week_1</t>
   </si>
@@ -243,6 +243,15 @@
   <si>
     <t>Services Page UI Connect with Services page and department pages (Controller + model)</t>
   </si>
+  <si>
+    <t>Implement Book Appointment Form functionality (Controller + Model + Route)</t>
+  </si>
+  <si>
+    <t>Create Appointments Database Table and connect form to MySQL</t>
+  </si>
+  <si>
+    <t>Improve Book Appointment UI and form validation</t>
+  </si>
 </sst>
 </file>
 
@@ -395,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="78">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -615,14 +624,8 @@
     <xf borderId="1" fillId="9" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="9" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="9" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -842,7 +845,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="10.0"/>
-    <col customWidth="1" min="2" max="2" width="67.5"/>
+    <col customWidth="1" min="2" max="2" width="80.63"/>
     <col customWidth="1" min="3" max="3" width="12.25"/>
     <col customWidth="1" min="4" max="4" width="12.13"/>
   </cols>
@@ -4236,10 +4239,16 @@
       <c r="AA100" s="3"/>
     </row>
     <row r="101">
-      <c r="A101" s="77"/>
-      <c r="B101" s="78"/>
-      <c r="C101" s="47"/>
-      <c r="D101" s="79"/>
+      <c r="A101" s="45"/>
+      <c r="B101" s="72" t="s">
+        <v>77</v>
+      </c>
+      <c r="C101" s="73">
+        <v>46090.0</v>
+      </c>
+      <c r="D101" s="77">
+        <v>2.25</v>
+      </c>
       <c r="E101" s="3"/>
       <c r="F101" s="3"/>
       <c r="G101" s="3"/>
@@ -4266,13 +4275,14 @@
     </row>
     <row r="102">
       <c r="A102" s="45"/>
-      <c r="B102" s="46" t="s">
-        <v>15</v>
+      <c r="B102" s="72" t="s">
+        <v>78</v>
       </c>
-      <c r="C102" s="47"/>
-      <c r="D102" s="41">
-        <f>sum(D91:D100)</f>
-        <v>22.7</v>
+      <c r="C102" s="73">
+        <v>46090.0</v>
+      </c>
+      <c r="D102" s="77">
+        <v>1.75</v>
       </c>
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
@@ -4299,10 +4309,16 @@
       <c r="AA102" s="3"/>
     </row>
     <row r="103">
-      <c r="A103" s="3"/>
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="D103" s="3"/>
+      <c r="A103" s="45"/>
+      <c r="B103" s="72" t="s">
+        <v>79</v>
+      </c>
+      <c r="C103" s="73">
+        <v>46090.0</v>
+      </c>
+      <c r="D103" s="77">
+        <v>1.0</v>
+      </c>
       <c r="E103" s="3"/>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
@@ -4328,10 +4344,15 @@
       <c r="AA103" s="3"/>
     </row>
     <row r="104">
-      <c r="A104" s="3"/>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
+      <c r="A104" s="45"/>
+      <c r="B104" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C104" s="47"/>
+      <c r="D104" s="41">
+        <f>sum(D91:D103)</f>
+        <v>27.7</v>
+      </c>
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
       <c r="G104" s="3"/>
@@ -29151,6 +29172,64 @@
       <c r="Z959" s="3"/>
       <c r="AA959" s="3"/>
     </row>
+    <row r="960">
+      <c r="A960" s="3"/>
+      <c r="B960" s="3"/>
+      <c r="C960" s="3"/>
+      <c r="D960" s="3"/>
+      <c r="E960" s="3"/>
+      <c r="F960" s="3"/>
+      <c r="G960" s="3"/>
+      <c r="H960" s="3"/>
+      <c r="I960" s="3"/>
+      <c r="J960" s="3"/>
+      <c r="K960" s="3"/>
+      <c r="L960" s="3"/>
+      <c r="M960" s="3"/>
+      <c r="N960" s="3"/>
+      <c r="O960" s="3"/>
+      <c r="P960" s="3"/>
+      <c r="Q960" s="3"/>
+      <c r="R960" s="3"/>
+      <c r="S960" s="3"/>
+      <c r="T960" s="3"/>
+      <c r="U960" s="3"/>
+      <c r="V960" s="3"/>
+      <c r="W960" s="3"/>
+      <c r="X960" s="3"/>
+      <c r="Y960" s="3"/>
+      <c r="Z960" s="3"/>
+      <c r="AA960" s="3"/>
+    </row>
+    <row r="961">
+      <c r="A961" s="3"/>
+      <c r="B961" s="3"/>
+      <c r="C961" s="3"/>
+      <c r="D961" s="3"/>
+      <c r="E961" s="3"/>
+      <c r="F961" s="3"/>
+      <c r="G961" s="3"/>
+      <c r="H961" s="3"/>
+      <c r="I961" s="3"/>
+      <c r="J961" s="3"/>
+      <c r="K961" s="3"/>
+      <c r="L961" s="3"/>
+      <c r="M961" s="3"/>
+      <c r="N961" s="3"/>
+      <c r="O961" s="3"/>
+      <c r="P961" s="3"/>
+      <c r="Q961" s="3"/>
+      <c r="R961" s="3"/>
+      <c r="S961" s="3"/>
+      <c r="T961" s="3"/>
+      <c r="U961" s="3"/>
+      <c r="V961" s="3"/>
+      <c r="W961" s="3"/>
+      <c r="X961" s="3"/>
+      <c r="Y961" s="3"/>
+      <c r="Z961" s="3"/>
+      <c r="AA961" s="3"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Modify CSS and fix error in pages
</commit_message>
<xml_diff>
--- a/Week_8/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_8/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="81">
   <si>
     <t>Week_1</t>
   </si>
@@ -251,6 +251,9 @@
   </si>
   <si>
     <t>Improve Book Appointment UI and form validation</t>
+  </si>
+  <si>
+    <t>Modified some Css &amp; Page in Portfolio</t>
   </si>
 </sst>
 </file>
@@ -4346,12 +4349,13 @@
     <row r="104">
       <c r="A104" s="45"/>
       <c r="B104" s="46" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
-      <c r="C104" s="47"/>
-      <c r="D104" s="41">
-        <f>sum(D91:D103)</f>
-        <v>27.7</v>
+      <c r="C104" s="73">
+        <v>46092.0</v>
+      </c>
+      <c r="D104" s="77">
+        <v>1.75</v>
       </c>
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
@@ -4378,10 +4382,15 @@
       <c r="AA104" s="3"/>
     </row>
     <row r="105">
-      <c r="A105" s="3"/>
-      <c r="B105" s="3"/>
-      <c r="C105" s="3"/>
-      <c r="D105" s="3"/>
+      <c r="A105" s="45"/>
+      <c r="B105" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C105" s="47"/>
+      <c r="D105" s="41">
+        <f>sum(D91:D104)</f>
+        <v>29.45</v>
+      </c>
       <c r="E105" s="3"/>
       <c r="F105" s="3"/>
       <c r="G105" s="3"/>
@@ -29230,6 +29239,35 @@
       <c r="Z961" s="3"/>
       <c r="AA961" s="3"/>
     </row>
+    <row r="962">
+      <c r="A962" s="3"/>
+      <c r="B962" s="3"/>
+      <c r="C962" s="3"/>
+      <c r="D962" s="3"/>
+      <c r="E962" s="3"/>
+      <c r="F962" s="3"/>
+      <c r="G962" s="3"/>
+      <c r="H962" s="3"/>
+      <c r="I962" s="3"/>
+      <c r="J962" s="3"/>
+      <c r="K962" s="3"/>
+      <c r="L962" s="3"/>
+      <c r="M962" s="3"/>
+      <c r="N962" s="3"/>
+      <c r="O962" s="3"/>
+      <c r="P962" s="3"/>
+      <c r="Q962" s="3"/>
+      <c r="R962" s="3"/>
+      <c r="S962" s="3"/>
+      <c r="T962" s="3"/>
+      <c r="U962" s="3"/>
+      <c r="V962" s="3"/>
+      <c r="W962" s="3"/>
+      <c r="X962" s="3"/>
+      <c r="Y962" s="3"/>
+      <c r="Z962" s="3"/>
+      <c r="AA962" s="3"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>